<commit_message>
Update P1 to the current flow package
Adds the two modules the September work lives in: integrity_fixes.py (exact
allow-list matching, retryPolicy placement, resume-save gating, deterministic
row pick, and the terminate/alert ordering fix) and reliability_flow.py, where
resume naming now derives from the target row so a resend replaces the
candidate's previous CV instead of adding a second file.

Also brings across the consolidated technical design document, the operator
runbook, the reviewed reply catalogue and the September 8 review evidence, and
refreshes the built definition, package zip, config and test suite. Suite at
797 passing.

Candidate data stays excluded; the committed workbook is an empty 33-column
schema template.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DriverAI_HiringAgent/HiringAgent_P1/P1_Templates/HiringAgent_P1_CandidateList.xlsx
+++ b/DriverAI_HiringAgent/HiringAgent_P1/P1_Templates/HiringAgent_P1_CandidateList.xlsx
@@ -126,9 +126,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HiringAgent_P1_Candidates" displayName="HiringAgent_P1_Candidates" ref="A1:AD2" headerRowCount="1">
-  <autoFilter ref="A1:AD2"/>
-  <tableColumns count="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="HiringAgent_P1_Candidates" displayName="HiringAgent_P1_Candidates" ref="A1:AG2" headerRowCount="1">
+  <tableColumns count="33">
     <tableColumn id="1" name="Application ID"/>
     <tableColumn id="2" name="Received Date"/>
     <tableColumn id="3" name="Last Updated Date"/>
@@ -139,35 +138,37 @@
     <tableColumn id="8" name="Phone"/>
     <tableColumn id="9" name="Location"/>
     <tableColumn id="10" name="Country"/>
-    <tableColumn id="11" name="Current Skills"/>
-    <tableColumn id="12" name="Education"/>
-    <tableColumn id="13" name="Looking For Role"/>
-    <tableColumn id="14" name="Suggested Role 1"/>
-    <tableColumn id="15" name="Suggested Role 2"/>
-    <tableColumn id="16" name="Suggested Role 3"/>
-    <tableColumn id="17" name="Mail Subject"/>
-    <tableColumn id="18" name="Mail Body"/>
-    <tableColumn id="19" name="Status"/>
-    <tableColumn id="20" name="Has Resume"/>
-    <tableColumn id="21" name="Original Filename"/>
-    <tableColumn id="22" name="Application Updates"/>
-    <tableColumn id="23" name="Retry Count"/>
-    <tableColumn id="24" name="Portfolio 1"/>
-    <tableColumn id="25" name="Portfolio 2"/>
-    <tableColumn id="26" name="Portfolio 3"/>
-    <tableColumn id="27" name="Resume URL"/>
-    <tableColumn id="28" name="Resume Folder Path"/>
-    <tableColumn id="29" name="Mail Sent"/>
-    <tableColumn id="30" name="Info Request Sent"/>
+    <tableColumn id="11" name="Years Exp"/>
+    <tableColumn id="12" name="Current Skills"/>
+    <tableColumn id="13" name="Education"/>
+    <tableColumn id="14" name="Education Start Date"/>
+    <tableColumn id="15" name="Education End Date"/>
+    <tableColumn id="16" name="Looking For Role"/>
+    <tableColumn id="17" name="Suggested Role 1"/>
+    <tableColumn id="18" name="Suggested Role 2"/>
+    <tableColumn id="19" name="Suggested Role 3"/>
+    <tableColumn id="20" name="Mail Subject"/>
+    <tableColumn id="21" name="Mail Body"/>
+    <tableColumn id="22" name="Status"/>
+    <tableColumn id="23" name="Has Resume"/>
+    <tableColumn id="24" name="Original Filename"/>
+    <tableColumn id="25" name="Application Updates"/>
+    <tableColumn id="26" name="Retry Count"/>
+    <tableColumn id="27" name="Portfolio 1"/>
+    <tableColumn id="28" name="Portfolio 2"/>
+    <tableColumn id="29" name="Portfolio 3"/>
+    <tableColumn id="30" name="Resume URL"/>
+    <tableColumn id="31" name="Resume Folder Path"/>
+    <tableColumn id="32" name="Mail Sent"/>
+    <tableColumn id="33" name="Info Request Sent"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="HiringAgent_P2_Rejected" displayName="HiringAgent_P2_Rejected" ref="A1:AC2" headerRowCount="1">
-  <autoFilter ref="A1:AC2"/>
-  <tableColumns count="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="HiringAgent_P2_Rejected" displayName="HiringAgent_P2_Rejected" ref="A1:AF2" headerRowCount="1">
+  <tableColumns count="32">
     <tableColumn id="1" name="Application ID"/>
     <tableColumn id="2" name="Received Date"/>
     <tableColumn id="3" name="Last Updated Date"/>
@@ -178,27 +179,30 @@
     <tableColumn id="8" name="Phone"/>
     <tableColumn id="9" name="Location"/>
     <tableColumn id="10" name="Country"/>
-    <tableColumn id="11" name="Current Skills"/>
-    <tableColumn id="12" name="Education"/>
-    <tableColumn id="13" name="Looking For Role"/>
-    <tableColumn id="14" name="Suggested Role 1"/>
-    <tableColumn id="15" name="Suggested Role 2"/>
-    <tableColumn id="16" name="Suggested Role 3"/>
-    <tableColumn id="17" name="Mail Subject"/>
-    <tableColumn id="18" name="Mail Body"/>
-    <tableColumn id="19" name="Status"/>
-    <tableColumn id="20" name="Has Resume"/>
-    <tableColumn id="21" name="Original Filename"/>
-    <tableColumn id="22" name="Application Updates"/>
-    <tableColumn id="23" name="Retry Count"/>
-    <tableColumn id="24" name="Portfolio 1"/>
-    <tableColumn id="25" name="Portfolio 2"/>
-    <tableColumn id="26" name="Portfolio 3"/>
-    <tableColumn id="27" name="Resume URL"/>
-    <tableColumn id="28" name="Resume Folder Path"/>
-    <tableColumn id="29" name="Decline Sent"/>
+    <tableColumn id="11" name="Years Exp"/>
+    <tableColumn id="12" name="Current Skills"/>
+    <tableColumn id="13" name="Education"/>
+    <tableColumn id="14" name="Education Start Date"/>
+    <tableColumn id="15" name="Education End Date"/>
+    <tableColumn id="16" name="Looking For Role"/>
+    <tableColumn id="17" name="Suggested Role 1"/>
+    <tableColumn id="18" name="Suggested Role 2"/>
+    <tableColumn id="19" name="Suggested Role 3"/>
+    <tableColumn id="20" name="Mail Subject"/>
+    <tableColumn id="21" name="Mail Body"/>
+    <tableColumn id="22" name="Status"/>
+    <tableColumn id="23" name="Has Resume"/>
+    <tableColumn id="24" name="Original Filename"/>
+    <tableColumn id="25" name="Application Updates"/>
+    <tableColumn id="26" name="Retry Count"/>
+    <tableColumn id="27" name="Portfolio 1"/>
+    <tableColumn id="28" name="Portfolio 2"/>
+    <tableColumn id="29" name="Portfolio 3"/>
+    <tableColumn id="30" name="Resume URL"/>
+    <tableColumn id="31" name="Resume Folder Path"/>
+    <tableColumn id="32" name="Decline Sent"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -491,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AG2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -547,100 +551,115 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Years Exp</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Current Skills</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Education Start Date</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Education End Date</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>Looking For Role</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Suggested Role 1</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Suggested Role 2</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Suggested Role 3</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Mail Subject</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Mail Body</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Has Resume</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Original Filename</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Application Updates</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Retry Count</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Portfolio 1</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Portfolio 2</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Portfolio 3</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Resume URL</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Resume Folder Path</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Mail Sent</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Info Request Sent</t>
         </is>
@@ -677,6 +696,9 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -692,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -748,95 +770,110 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Years Exp</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Current Skills</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Education Start Date</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Education End Date</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>Looking For Role</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Suggested Role 1</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Suggested Role 2</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Suggested Role 3</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Mail Subject</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Mail Body</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Has Resume</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Original Filename</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Application Updates</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Retry Count</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Portfolio 1</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Portfolio 2</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Portfolio 3</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Resume URL</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Resume Folder Path</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Decline Sent</t>
         </is>
@@ -872,6 +909,9 @@
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>